<commit_message>
Update attendees for quiz: mongodb-training — anburajs@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -455,9 +455,50 @@
         <v>Grade</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>anburajs@clarium.tech</v>
+      </c>
+      <c r="B2" t="str">
+        <v>anburaj selvaraj</v>
+      </c>
+      <c r="C2" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D2" t="str">
+        <v>3/27/2026, 4:04:59 PM</v>
+      </c>
+      <c r="E2">
+        <v>25</v>
+      </c>
+      <c r="F2">
+        <v>25</v>
+      </c>
+      <c r="G2">
+        <v>17</v>
+      </c>
+      <c r="H2">
+        <v>8</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>41</v>
+      </c>
+      <c r="K2">
+        <v>25</v>
+      </c>
+      <c r="L2" t="str">
+        <v>60.98</v>
+      </c>
+      <c r="M2" t="str">
+        <v>C</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — charanm@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -496,9 +496,50 @@
         <v>C</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>charanm@clarium.tech</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Charan M</v>
+      </c>
+      <c r="C3" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D3" t="str">
+        <v>3/27/2026, 4:05:57 PM</v>
+      </c>
+      <c r="E3">
+        <v>25</v>
+      </c>
+      <c r="F3">
+        <v>25</v>
+      </c>
+      <c r="G3">
+        <v>21</v>
+      </c>
+      <c r="H3">
+        <v>4</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>41</v>
+      </c>
+      <c r="K3">
+        <v>32</v>
+      </c>
+      <c r="L3" t="str">
+        <v>78.05</v>
+      </c>
+      <c r="M3" t="str">
+        <v>B</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — ramagurua@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -537,9 +537,50 @@
         <v>B</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ramagurua@clarium.tech</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Ramaguru</v>
+      </c>
+      <c r="C4" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D4" t="str">
+        <v>3/27/2026, 4:06:27 PM</v>
+      </c>
+      <c r="E4">
+        <v>25</v>
+      </c>
+      <c r="F4">
+        <v>25</v>
+      </c>
+      <c r="G4">
+        <v>13</v>
+      </c>
+      <c r="H4">
+        <v>12</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>41</v>
+      </c>
+      <c r="K4">
+        <v>20</v>
+      </c>
+      <c r="L4" t="str">
+        <v>48.78</v>
+      </c>
+      <c r="M4" t="str">
+        <v>F</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — jayarajr@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -578,9 +578,50 @@
         <v>F</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>jayarajr@clarium.tech</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Jayaraj Raja</v>
+      </c>
+      <c r="C5" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D5" t="str">
+        <v>3/27/2026, 4:06:29 PM</v>
+      </c>
+      <c r="E5">
+        <v>25</v>
+      </c>
+      <c r="F5">
+        <v>25</v>
+      </c>
+      <c r="G5">
+        <v>18</v>
+      </c>
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>41</v>
+      </c>
+      <c r="K5">
+        <v>28</v>
+      </c>
+      <c r="L5" t="str">
+        <v>68.29</v>
+      </c>
+      <c r="M5" t="str">
+        <v>C</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — veeraragavans@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -619,9 +619,50 @@
         <v>C</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>veeraragavans@clarium.tech</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Veeraragavan</v>
+      </c>
+      <c r="C6" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D6" t="str">
+        <v>3/27/2026, 4:06:33 PM</v>
+      </c>
+      <c r="E6">
+        <v>25</v>
+      </c>
+      <c r="F6">
+        <v>25</v>
+      </c>
+      <c r="G6">
+        <v>19</v>
+      </c>
+      <c r="H6">
+        <v>6</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>41</v>
+      </c>
+      <c r="K6">
+        <v>30</v>
+      </c>
+      <c r="L6" t="str">
+        <v>73.17</v>
+      </c>
+      <c r="M6" t="str">
+        <v>B</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — vivekkumarsps@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D2" t="str">
-        <v>3/27/2026, 4:04:59 PM</v>
+        <v>27/3/2026, 4:04:59 pm</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D3" t="str">
-        <v>3/27/2026, 4:05:57 PM</v>
+        <v>27/3/2026, 4:05:57 pm</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D4" t="str">
-        <v>3/27/2026, 4:06:27 PM</v>
+        <v>27/3/2026, 4:06:27 pm</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D5" t="str">
-        <v>3/27/2026, 4:06:29 PM</v>
+        <v>27/3/2026, 4:06:29 pm</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D6" t="str">
-        <v>3/27/2026, 4:06:33 PM</v>
+        <v>27/3/2026, 4:06:33 pm</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -658,11 +658,52 @@
       </c>
       <c r="M6" t="str">
         <v>B</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>vivekkumarsps@clarium.tech</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Vivek Kumar Singh</v>
+      </c>
+      <c r="C7" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D7" t="str">
+        <v>27/3/2026, 4:06:50 pm</v>
+      </c>
+      <c r="E7">
+        <v>25</v>
+      </c>
+      <c r="F7">
+        <v>25</v>
+      </c>
+      <c r="G7">
+        <v>17</v>
+      </c>
+      <c r="H7">
+        <v>8</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>41</v>
+      </c>
+      <c r="K7">
+        <v>26</v>
+      </c>
+      <c r="L7" t="str">
+        <v>63.41</v>
+      </c>
+      <c r="M7" t="str">
+        <v>C</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — himabindus@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D2" t="str">
-        <v>27/3/2026, 4:04:59 pm</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D3" t="str">
-        <v>27/3/2026, 4:05:57 pm</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D4" t="str">
-        <v>27/3/2026, 4:06:27 pm</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D5" t="str">
-        <v>27/3/2026, 4:06:29 pm</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D6" t="str">
-        <v>27/3/2026, 4:06:33 pm</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -671,7 +671,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D7" t="str">
-        <v>27/3/2026, 4:06:50 pm</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E7">
         <v>25</v>
@@ -699,11 +699,52 @@
       </c>
       <c r="M7" t="str">
         <v>C</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>himabindus@clarium.tech</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Himabindu Mallarapu</v>
+      </c>
+      <c r="C8" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D8" t="str">
+        <v>27/3/2026, 4:07:04 pm</v>
+      </c>
+      <c r="E8">
+        <v>25</v>
+      </c>
+      <c r="F8">
+        <v>25</v>
+      </c>
+      <c r="G8">
+        <v>19</v>
+      </c>
+      <c r="H8">
+        <v>6</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>41</v>
+      </c>
+      <c r="K8">
+        <v>29</v>
+      </c>
+      <c r="L8" t="str">
+        <v>70.73</v>
+      </c>
+      <c r="M8" t="str">
+        <v>B</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — keerthivasanp@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -712,7 +712,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D8" t="str">
-        <v>27/3/2026, 4:07:04 pm</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E8">
         <v>25</v>
@@ -742,9 +742,50 @@
         <v>B</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>keerthivasanp@clarium.tech</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Keerthi Vasan</v>
+      </c>
+      <c r="C9" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D9" t="str">
+        <v>27/3/2026, 4:07:28 pm</v>
+      </c>
+      <c r="E9">
+        <v>25</v>
+      </c>
+      <c r="F9">
+        <v>25</v>
+      </c>
+      <c r="G9">
+        <v>23</v>
+      </c>
+      <c r="H9">
+        <v>2</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>41</v>
+      </c>
+      <c r="K9">
+        <v>37</v>
+      </c>
+      <c r="L9" t="str">
+        <v>90.24</v>
+      </c>
+      <c r="M9" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — vinayagams@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -753,7 +753,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D9" t="str">
-        <v>27/3/2026, 4:07:28 pm</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E9">
         <v>25</v>
@@ -783,9 +783,50 @@
         <v>A+</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>vinayagams@clarium.tech</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Vinayagam</v>
+      </c>
+      <c r="C10" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D10" t="str">
+        <v>3/27/2026, 4:07:55 PM</v>
+      </c>
+      <c r="E10">
+        <v>25</v>
+      </c>
+      <c r="F10">
+        <v>25</v>
+      </c>
+      <c r="G10">
+        <v>19</v>
+      </c>
+      <c r="H10">
+        <v>6</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>41</v>
+      </c>
+      <c r="K10">
+        <v>30</v>
+      </c>
+      <c r="L10" t="str">
+        <v>73.17</v>
+      </c>
+      <c r="M10" t="str">
+        <v>B</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — ramua@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -794,7 +794,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D10" t="str">
-        <v>3/27/2026, 4:07:55 PM</v>
+        <v>27/3/2026, 4:07:55 pm</v>
       </c>
       <c r="E10">
         <v>25</v>
@@ -824,9 +824,50 @@
         <v>B</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>ramua@clarium.tech</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Ramu A</v>
+      </c>
+      <c r="C11" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D11" t="str">
+        <v>27/3/2026, 4:09:20 pm</v>
+      </c>
+      <c r="E11">
+        <v>25</v>
+      </c>
+      <c r="F11">
+        <v>25</v>
+      </c>
+      <c r="G11">
+        <v>23</v>
+      </c>
+      <c r="H11">
+        <v>2</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>41</v>
+      </c>
+      <c r="K11">
+        <v>37</v>
+      </c>
+      <c r="L11" t="str">
+        <v>90.24</v>
+      </c>
+      <c r="M11" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — nanneelanc@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -794,7 +794,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D10" t="str">
-        <v>27/3/2026, 4:07:55 pm</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E10">
         <v>25</v>
@@ -835,7 +835,7 @@
         <v>MongoDB Training</v>
       </c>
       <c r="D11" t="str">
-        <v>27/3/2026, 4:09:20 pm</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E11">
         <v>25</v>
@@ -865,9 +865,50 @@
         <v>A+</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>nanneelanc@clarium.tech</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Nanneelan Chinnamuthu</v>
+      </c>
+      <c r="C12" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D12" t="str">
+        <v>3/27/2026, 4:09:59 PM</v>
+      </c>
+      <c r="E12">
+        <v>25</v>
+      </c>
+      <c r="F12">
+        <v>25</v>
+      </c>
+      <c r="G12">
+        <v>20</v>
+      </c>
+      <c r="H12">
+        <v>5</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>41</v>
+      </c>
+      <c r="K12">
+        <v>33</v>
+      </c>
+      <c r="L12" t="str">
+        <v>80.49</v>
+      </c>
+      <c r="M12" t="str">
+        <v>A</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — sanepayiabdullateefmp@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -906,9 +906,50 @@
         <v>A</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>sanepayiabdullateefmp@clarium.tech</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Abdul Lateef</v>
+      </c>
+      <c r="C13" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D13" t="str">
+        <v>3/27/2026, 4:10:26 PM</v>
+      </c>
+      <c r="E13">
+        <v>25</v>
+      </c>
+      <c r="F13">
+        <v>25</v>
+      </c>
+      <c r="G13">
+        <v>21</v>
+      </c>
+      <c r="H13">
+        <v>4</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>41</v>
+      </c>
+      <c r="K13">
+        <v>33</v>
+      </c>
+      <c r="L13" t="str">
+        <v>80.49</v>
+      </c>
+      <c r="M13" t="str">
+        <v>A</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — nobelfranklinl@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M14"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -947,9 +947,50 @@
         <v>A</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>nobelfranklinl@clarium.tech</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Nobe Franklin</v>
+      </c>
+      <c r="C14" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D14" t="str">
+        <v>3/27/2026, 4:10:33 PM</v>
+      </c>
+      <c r="E14">
+        <v>25</v>
+      </c>
+      <c r="F14">
+        <v>25</v>
+      </c>
+      <c r="G14">
+        <v>24</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>41</v>
+      </c>
+      <c r="K14">
+        <v>38</v>
+      </c>
+      <c r="L14" t="str">
+        <v>92.68</v>
+      </c>
+      <c r="M14" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — bharathm@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -988,9 +988,50 @@
         <v>A+</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>bharathm@clarium.tech</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Bharath</v>
+      </c>
+      <c r="C15" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D15" t="str">
+        <v>3/27/2026, 4:10:57 PM</v>
+      </c>
+      <c r="E15">
+        <v>25</v>
+      </c>
+      <c r="F15">
+        <v>25</v>
+      </c>
+      <c r="G15">
+        <v>18</v>
+      </c>
+      <c r="H15">
+        <v>7</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>41</v>
+      </c>
+      <c r="K15">
+        <v>29</v>
+      </c>
+      <c r="L15" t="str">
+        <v>70.73</v>
+      </c>
+      <c r="M15" t="str">
+        <v>B</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — gokuls@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M16"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -1029,9 +1029,50 @@
         <v>B</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>gokuls@clarium.tech</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Gokul</v>
+      </c>
+      <c r="C16" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D16" t="str">
+        <v>3/27/2026, 4:11:51 PM</v>
+      </c>
+      <c r="E16">
+        <v>25</v>
+      </c>
+      <c r="F16">
+        <v>25</v>
+      </c>
+      <c r="G16">
+        <v>18</v>
+      </c>
+      <c r="H16">
+        <v>7</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>41</v>
+      </c>
+      <c r="K16">
+        <v>28</v>
+      </c>
+      <c r="L16" t="str">
+        <v>68.29</v>
+      </c>
+      <c r="M16" t="str">
+        <v>C</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — dineshag@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M17"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -1070,9 +1070,50 @@
         <v>C</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>dineshag@clarium.tech</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Dinesha Gunasekaran</v>
+      </c>
+      <c r="C17" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D17" t="str">
+        <v>3/27/2026, 4:11:58 PM</v>
+      </c>
+      <c r="E17">
+        <v>25</v>
+      </c>
+      <c r="F17">
+        <v>25</v>
+      </c>
+      <c r="G17">
+        <v>24</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>41</v>
+      </c>
+      <c r="K17">
+        <v>40</v>
+      </c>
+      <c r="L17" t="str">
+        <v>97.56</v>
+      </c>
+      <c r="M17" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-training — deepakk@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-training/attendees.xlsx
+++ b/quizzes/mongodb-training/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M18"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -1111,9 +1111,50 @@
         <v>A+</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>deepakk@clarium.tech</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Deepak</v>
+      </c>
+      <c r="C18" t="str">
+        <v>MongoDB Training</v>
+      </c>
+      <c r="D18" t="str">
+        <v>3/27/2026, 4:13:11 PM</v>
+      </c>
+      <c r="E18">
+        <v>25</v>
+      </c>
+      <c r="F18">
+        <v>25</v>
+      </c>
+      <c r="G18">
+        <v>20</v>
+      </c>
+      <c r="H18">
+        <v>5</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>41</v>
+      </c>
+      <c r="K18">
+        <v>32</v>
+      </c>
+      <c r="L18" t="str">
+        <v>78.05</v>
+      </c>
+      <c r="M18" t="str">
+        <v>B</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>